<commit_message>
Add character graphics rendering
</commit_message>
<xml_diff>
--- a/segments.xlsx
+++ b/segments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dom.cresswell/Dropbox/Geek/Gaming Projects/Bloodwych 68k/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD68388-4CF4-C749-BD3E-EF9941A14933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE34092-C3AE-DF40-9D20-9041A28DC93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="400" yWindow="880" windowWidth="29460" windowHeight="21620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3720" yWindow="880" windowWidth="29460" windowHeight="21620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BLOODWYCH439" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7748" uniqueCount="3834">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7797" uniqueCount="3882">
   <si>
     <t>Type</t>
   </si>
@@ -11539,6 +11539,150 @@
   </si>
   <si>
     <t>Offsets for the Crab body, face, front, back, and side components across Crab.gfx and CrabClaw.gfx.</t>
+  </si>
+  <si>
+    <t>Character_BodyDefinitions</t>
+  </si>
+  <si>
+    <t>characters-body-definitions.layout</t>
+  </si>
+  <si>
+    <t>$A50A</t>
+  </si>
+  <si>
+    <t>8C</t>
+  </si>
+  <si>
+    <t>Character_PartFacingVariants</t>
+  </si>
+  <si>
+    <t>characters-part-variants.lookup</t>
+  </si>
+  <si>
+    <t>data/characters-part-variants.lookup</t>
+  </si>
+  <si>
+    <t>$A600</t>
+  </si>
+  <si>
+    <t>Character_RenderTableOffsets</t>
+  </si>
+  <si>
+    <t>characters-render-table-offsets.lookup</t>
+  </si>
+  <si>
+    <t>data/characters-render-table-offsets.lookup</t>
+  </si>
+  <si>
+    <t>$A5EC</t>
+  </si>
+  <si>
+    <t>Character_ArmAnimationPositions</t>
+  </si>
+  <si>
+    <t>characters-arm-animation.positions</t>
+  </si>
+  <si>
+    <t>data/characters-arm-animation.positions</t>
+  </si>
+  <si>
+    <t>$A778</t>
+  </si>
+  <si>
+    <t>Character_RenderLayout_Standard</t>
+  </si>
+  <si>
+    <t>characters-standard-render.layout</t>
+  </si>
+  <si>
+    <t>data/characters-standard-render.layout</t>
+  </si>
+  <si>
+    <t>$18480</t>
+  </si>
+  <si>
+    <t>Character_Distant4_Positions_Standard</t>
+  </si>
+  <si>
+    <t>characters-standard-distant-4.positions</t>
+  </si>
+  <si>
+    <t>data/characters-standard-distant-4.positions</t>
+  </si>
+  <si>
+    <t>$185B0</t>
+  </si>
+  <si>
+    <t>Character_Distant5_Positions_Standard</t>
+  </si>
+  <si>
+    <t>characters-standard-distant-5.positions</t>
+  </si>
+  <si>
+    <t>data/characters-standard-distant-5.positions</t>
+  </si>
+  <si>
+    <t>$185B8</t>
+  </si>
+  <si>
+    <t>Character_RenderLayout_Alternate</t>
+  </si>
+  <si>
+    <t>characters-alternate-render.layout</t>
+  </si>
+  <si>
+    <t>data/characters-alternate-render.layout</t>
+  </si>
+  <si>
+    <t>$185C0</t>
+  </si>
+  <si>
+    <t>Character_Distant4_Positions_Alternate</t>
+  </si>
+  <si>
+    <t>characters-alternate-distant-4.positions</t>
+  </si>
+  <si>
+    <t>data/characters-alternate-distant-4.positions</t>
+  </si>
+  <si>
+    <t>$186F0</t>
+  </si>
+  <si>
+    <t>Character_Distant5_Positions_Alternate</t>
+  </si>
+  <si>
+    <t>characters-alternate-distant-5.positions</t>
+  </si>
+  <si>
+    <t>data/characters-alternate-distant-5.positions</t>
+  </si>
+  <si>
+    <t>$186F8</t>
+  </si>
+  <si>
+    <t>Draw_CharacterComponent</t>
+  </si>
+  <si>
+    <t>Fourteen 10-byte records containing a layout selector and BodyParts.gfx bases for legs, torso, arms and the distant composite.</t>
+  </si>
+  <si>
+    <t>Four signed XY pairs for the corresponding distant graphics slot.</t>
+  </si>
+  <si>
+    <t>Standard and alternate animated-arm Y corrections and facing-specific X corrections.</t>
+  </si>
+  <si>
+    <t>Five parts × four facings; bit 7 means mirror and $FF suppresses that part.</t>
+  </si>
+  <si>
+    <t>Interleaved five-entry lookup containing the height-table and graphics-source-table offsets for each rendered character part.</t>
+  </si>
+  <si>
+    <t>_Offset_Character_RenderTableOffsets_0x02</t>
+  </si>
+  <si>
+    <t>Draws one character component by selecting its distance, facing and animation variant, resolving its height and graphics source, applying its colour mask, and positioning or mirroring the 16-pixel strip.</t>
   </si>
 </sst>
 </file>
@@ -11719,7 +11863,64 @@
     <cellStyle name="Excel Built-in Normal" xfId="1" xr:uid="{ACE51F02-8306-284E-B6CB-6CB2D79D3F1F}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="3" tint="0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.749961851863155"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="5" tint="-0.24994659260841701"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="3" tint="0.24994659260841701"/>
@@ -12117,7 +12318,8 @@
     <col min="5" max="5" width="61.5" customWidth="1"/>
     <col min="6" max="6" width="19.5" customWidth="1"/>
     <col min="7" max="8" width="10.83203125" style="5" customWidth="1"/>
-    <col min="9" max="10" width="14.83203125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" style="6" customWidth="1"/>
+    <col min="10" max="10" width="26.83203125" style="6" customWidth="1"/>
     <col min="11" max="11" width="103.33203125" style="6" bestFit="1" customWidth="1"/>
     <col min="12" max="13" width="14.83203125" style="6" customWidth="1"/>
     <col min="14" max="15" width="70.83203125" customWidth="1"/>
@@ -19502,7 +19704,7 @@
         <v>3813</v>
       </c>
     </row>
-    <row r="210" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:11" ht="17" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>3342</v>
       </c>
@@ -19531,7 +19733,7 @@
       <c r="J210" s="6" t="s">
         <v>3657</v>
       </c>
-      <c r="K210" t="s">
+      <c r="K210" s="26" t="s">
         <v>3814</v>
       </c>
     </row>
@@ -57233,76 +57435,143 @@
         <v>321</v>
       </c>
     </row>
-    <row r="2134" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2134" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2134" t="s">
         <v>2419</v>
       </c>
-      <c r="B2134" t="s">
-        <v>321</v>
+      <c r="B2134" s="26" t="s">
+        <v>3834</v>
+      </c>
+      <c r="C2134" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2134" s="26" t="s">
+        <v>3835</v>
       </c>
       <c r="E2134" t="str">
         <f t="shared" si="64"/>
-        <v/>
+        <v>data/characters-body-definitions.layout</v>
+      </c>
+      <c r="F2134" t="s">
+        <v>3836</v>
+      </c>
+      <c r="G2134">
+        <v>42250</v>
+      </c>
+      <c r="H2134">
+        <v>140</v>
+      </c>
+      <c r="I2134" s="26" t="s">
+        <v>3837</v>
+      </c>
+      <c r="K2134" s="6" t="s">
+        <v>3875</v>
       </c>
       <c r="O2134" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2135" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2135" t="s">
+    <row r="2135" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2135" s="26" t="s">
         <v>2421</v>
       </c>
-      <c r="B2135" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2135" t="str">
-        <f t="shared" si="64"/>
-        <v/>
+      <c r="B2135" s="26" t="s">
+        <v>3842</v>
+      </c>
+      <c r="C2135" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2135" s="26" t="s">
+        <v>3843</v>
+      </c>
+      <c r="E2135" s="26" t="s">
+        <v>3844</v>
+      </c>
+      <c r="F2135" t="s">
+        <v>3845</v>
+      </c>
+      <c r="G2135">
+        <v>42476</v>
+      </c>
+      <c r="H2135">
+        <v>20</v>
+      </c>
+      <c r="I2135" s="26">
+        <v>14</v>
+      </c>
+      <c r="J2135"/>
+      <c r="K2135" t="s">
+        <v>3879</v>
       </c>
       <c r="O2135" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2136" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2136" t="s">
+    <row r="2136" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2136" s="26" t="s">
         <v>2422</v>
       </c>
-      <c r="B2136" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2136" t="str">
-        <f t="shared" si="64"/>
-        <v/>
-      </c>
+      <c r="B2136" s="26" t="s">
+        <v>3880</v>
+      </c>
+      <c r="C2136"/>
+      <c r="G2136"/>
+      <c r="H2136"/>
+      <c r="I2136"/>
+      <c r="J2136"/>
+      <c r="K2136"/>
       <c r="O2136" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2137" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2137" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2137" t="s">
         <v>2423</v>
       </c>
-      <c r="B2137" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2137" t="str">
-        <f t="shared" si="64"/>
-        <v/>
+      <c r="B2137" s="26" t="s">
+        <v>3838</v>
+      </c>
+      <c r="C2137" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2137" s="26" t="s">
+        <v>3839</v>
+      </c>
+      <c r="E2137" s="26" t="s">
+        <v>3840</v>
+      </c>
+      <c r="F2137" t="s">
+        <v>3841</v>
+      </c>
+      <c r="G2137">
+        <v>42496</v>
+      </c>
+      <c r="H2137">
+        <v>20</v>
+      </c>
+      <c r="I2137" s="26">
+        <v>14</v>
+      </c>
+      <c r="K2137" s="6" t="s">
+        <v>3878</v>
       </c>
       <c r="O2137" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2138" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2138" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2138" t="s">
         <v>2424</v>
       </c>
-      <c r="B2138" t="s">
-        <v>321</v>
+      <c r="B2138" s="26" t="s">
+        <v>3874</v>
       </c>
       <c r="E2138" t="str">
         <f t="shared" si="64"/>
         <v/>
+      </c>
+      <c r="K2138" s="6" t="s">
+        <v>3881</v>
       </c>
       <c r="O2138" t="s">
         <v>321</v>
@@ -57518,16 +57787,36 @@
         <v>321</v>
       </c>
     </row>
-    <row r="2153" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2153" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2153" t="s">
         <v>2439</v>
       </c>
-      <c r="B2153" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2153" t="str">
-        <f t="shared" si="64"/>
-        <v/>
+      <c r="B2153" s="26" t="s">
+        <v>3846</v>
+      </c>
+      <c r="C2153" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2153" s="26" t="s">
+        <v>3847</v>
+      </c>
+      <c r="E2153" s="26" t="s">
+        <v>3848</v>
+      </c>
+      <c r="F2153" t="s">
+        <v>3849</v>
+      </c>
+      <c r="G2153">
+        <v>42872</v>
+      </c>
+      <c r="H2153">
+        <v>72</v>
+      </c>
+      <c r="I2153" s="26">
+        <v>48</v>
+      </c>
+      <c r="K2153" s="6" t="s">
+        <v>3877</v>
       </c>
       <c r="O2153" t="s">
         <v>321</v>
@@ -64809,91 +65098,205 @@
         <v>3198</v>
       </c>
     </row>
-    <row r="2642" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2642" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2642" t="s">
         <v>3017</v>
       </c>
-      <c r="B2642" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2642" t="str">
-        <f t="shared" si="77"/>
-        <v/>
+      <c r="B2642" s="26" t="s">
+        <v>3850</v>
+      </c>
+      <c r="C2642" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2642" s="26" t="s">
+        <v>3851</v>
+      </c>
+      <c r="E2642" s="26" t="s">
+        <v>3852</v>
+      </c>
+      <c r="F2642" s="26" t="s">
+        <v>3853</v>
+      </c>
+      <c r="G2642">
+        <v>99456</v>
+      </c>
+      <c r="H2642">
+        <v>304</v>
+      </c>
+      <c r="I2642" s="26">
+        <v>130</v>
       </c>
       <c r="O2642" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2643" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2643" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2643" t="s">
         <v>3018</v>
       </c>
-      <c r="B2643" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2643" t="str">
-        <f t="shared" si="77"/>
-        <v/>
+      <c r="B2643" s="26" t="s">
+        <v>3854</v>
+      </c>
+      <c r="C2643" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2643" s="26" t="s">
+        <v>3855</v>
+      </c>
+      <c r="E2643" s="26" t="s">
+        <v>3856</v>
+      </c>
+      <c r="F2643" s="26" t="s">
+        <v>3857</v>
+      </c>
+      <c r="G2643">
+        <v>99760</v>
+      </c>
+      <c r="H2643">
+        <v>8</v>
+      </c>
+      <c r="I2643" s="26">
+        <v>8</v>
+      </c>
+      <c r="K2643" s="6" t="s">
+        <v>3876</v>
       </c>
       <c r="O2643" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2644" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2644" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2644" t="s">
         <v>3019</v>
       </c>
-      <c r="B2644" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2644" t="str">
-        <f t="shared" si="77"/>
-        <v/>
+      <c r="B2644" s="26" t="s">
+        <v>3858</v>
+      </c>
+      <c r="C2644" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2644" s="26" t="s">
+        <v>3859</v>
+      </c>
+      <c r="E2644" s="26" t="s">
+        <v>3860</v>
+      </c>
+      <c r="F2644" s="26" t="s">
+        <v>3861</v>
+      </c>
+      <c r="G2644">
+        <v>99768</v>
+      </c>
+      <c r="H2644">
+        <v>8</v>
+      </c>
+      <c r="I2644" s="26">
+        <v>8</v>
+      </c>
+      <c r="K2644" s="6" t="s">
+        <v>3876</v>
       </c>
       <c r="O2644" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2645" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2645" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2645" t="s">
         <v>3020</v>
       </c>
-      <c r="B2645" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2645" t="str">
-        <f t="shared" si="77"/>
-        <v/>
+      <c r="B2645" s="26" t="s">
+        <v>3862</v>
+      </c>
+      <c r="C2645" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2645" s="26" t="s">
+        <v>3863</v>
+      </c>
+      <c r="E2645" s="26" t="s">
+        <v>3864</v>
+      </c>
+      <c r="F2645" s="26" t="s">
+        <v>3865</v>
+      </c>
+      <c r="G2645">
+        <v>99776</v>
+      </c>
+      <c r="H2645">
+        <v>304</v>
+      </c>
+      <c r="I2645" s="26">
+        <v>130</v>
       </c>
       <c r="O2645" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2646" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2646" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2646" t="s">
         <v>3021</v>
       </c>
-      <c r="B2646" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2646" t="str">
-        <f t="shared" si="77"/>
-        <v/>
+      <c r="B2646" s="26" t="s">
+        <v>3866</v>
+      </c>
+      <c r="C2646" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2646" s="26" t="s">
+        <v>3867</v>
+      </c>
+      <c r="E2646" s="26" t="s">
+        <v>3868</v>
+      </c>
+      <c r="F2646" s="26" t="s">
+        <v>3869</v>
+      </c>
+      <c r="G2646">
+        <v>100080</v>
+      </c>
+      <c r="H2646">
+        <v>8</v>
+      </c>
+      <c r="I2646" s="26">
+        <v>8</v>
+      </c>
+      <c r="K2646" s="6" t="s">
+        <v>3876</v>
       </c>
       <c r="O2646" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2647" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2647" spans="1:15" ht="17" x14ac:dyDescent="0.25">
       <c r="A2647" t="s">
         <v>3022</v>
       </c>
-      <c r="B2647" t="s">
-        <v>321</v>
-      </c>
-      <c r="E2647" t="str">
-        <f t="shared" si="77"/>
-        <v/>
+      <c r="B2647" s="26" t="s">
+        <v>3870</v>
+      </c>
+      <c r="C2647" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2647" s="26" t="s">
+        <v>3871</v>
+      </c>
+      <c r="E2647" s="26" t="s">
+        <v>3872</v>
+      </c>
+      <c r="F2647" s="26" t="s">
+        <v>3873</v>
+      </c>
+      <c r="G2647">
+        <v>100088</v>
+      </c>
+      <c r="H2647">
+        <v>8</v>
+      </c>
+      <c r="I2647" s="26">
+        <v>8</v>
+      </c>
+      <c r="K2647" s="6" t="s">
+        <v>3876</v>
       </c>
       <c r="O2647" t="s">
         <v>321</v>
@@ -64974,30 +65377,28 @@
   </sheetData>
   <autoFilter ref="A1:R2651" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A2:A2651 A2695:A1048576">
-    <cfRule type="expression" dxfId="5" priority="13">
-      <formula>AND(MATCH(A2,A:A,0)=ROW(A2),COUNTIF(A:A,A2)=1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="14">
-      <formula>AND(MATCH(A2,A:A,0)=ROW(A2),COUNTIF(A:A,A2)&gt;1)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="17">
-      <formula>MATCH(A2,A:A,0)&lt;&gt;ROW(A2)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B200 B2695:B1048576 B205:B218 B221:B222 B229:B2651">
-    <cfRule type="expression" dxfId="2" priority="5">
+  <conditionalFormatting sqref="B2:B9998">
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>AND(B2&lt;&gt;"",_xlfn.ISFORMULA(B2)=TRUE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2695:O1048576 N55:O60 B193:D199 B188:B192 D188:D190 B200 D200:D202 B176:D187 B2:O36 F37:O54 F55:I60 B37:E175 B205:D218 F61:O187 E176:E2651 C203:C204 B221:D222 C219:C220 B229:D2651 C223:C228 F230:O2651 F188:J229 L188:O229">
-    <cfRule type="expression" dxfId="1" priority="6">
+  <conditionalFormatting sqref="B2:Z9998">
+    <cfRule type="expression" dxfId="4" priority="6">
       <formula>LEFT(LOWER($B2),7)="_delete"</formula>
     </cfRule>
+    <cfRule type="expression" dxfId="3" priority="12">
+      <formula>LEFT(LOWER($B2),7)="_offset"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N55:O60 B2695:O1048576 B193:D199 B188:B192 D188:D190 B200 D200:D202 B176:D187 B2:O36 F37:O54 F55:I60 B37:E175 B205:D218 F61:O187 E176:E2651 C203:C204 B221:D222 C219:C220 B229:D2651 C223:C228 F230:O2651 F188:J229 L188:O229">
-    <cfRule type="expression" dxfId="0" priority="12">
-      <formula>LEFT(LOWER($B2),7)="_offset"</formula>
+  <conditionalFormatting sqref="A2:A9998">
+    <cfRule type="expression" dxfId="2" priority="13">
+      <formula>AND(MATCH(A2,A:A,0)=ROW(A2),COUNTIF(A:A,A2)=1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="14">
+      <formula>AND(MATCH(A2,A:A,0)=ROW(A2),COUNTIF(A:A,A2)&gt;1)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="17" stopIfTrue="1">
+      <formula>MATCH(A2,A:A,0)&lt;&gt;ROW(A2)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>